<commit_message>
Align workbook outputs with notebook
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/magic_kitchens_analysis.xlsx
+++ b/output/magic_kitchens_analysis.xlsx
@@ -1862,7 +1862,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>★ RECOMMENDATION: Advertising (+$5.41K net) &gt; Promotion (+$3.10K net)</t>
+          <t>Q1 — $1K Recommendation: ADVERTISE (net +$5.41K) &gt; Promote (net +$3.10K)</t>
         </is>
       </c>
       <c r="C3" s="11" t="inlineStr">
@@ -2077,13 +2077,13 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>540.1900000000001</v>
+        <v>531.9400000000001</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>12.77</v>
+        <v>10.64</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>29.8</v>
+        <v>31.93</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>42.57</v>
@@ -2101,13 +2101,13 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>428.38</v>
+        <v>433.31</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>12.77</v>
+        <v>10.64</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>29.8</v>
+        <v>31.93</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>42.57</v>
@@ -2125,13 +2125,13 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>436.97</v>
+        <v>441.9</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>12.77</v>
+        <v>10.64</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>29.8</v>
+        <v>31.93</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>42.57</v>
@@ -2149,13 +2149,13 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>489.62</v>
+        <v>494.55</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>12.77</v>
+        <v>10.64</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>29.8</v>
+        <v>31.93</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>42.57</v>
@@ -2173,13 +2173,13 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>606.12</v>
+        <v>614.36</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>29.8</v>
+        <v>31.93</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>12.77</v>
+        <v>10.64</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>42.57</v>
@@ -2197,13 +2197,13 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>388.98</v>
+        <v>384.05</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>29.8</v>
+        <v>31.93</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>12.77</v>
+        <v>10.64</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>42.57</v>
@@ -2221,13 +2221,13 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>397.57</v>
+        <v>392.64</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>29.8</v>
+        <v>31.93</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>12.77</v>
+        <v>10.64</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>42.57</v>
@@ -2245,13 +2245,13 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>450.22</v>
+        <v>445.29</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>29.8</v>
+        <v>31.93</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>12.77</v>
+        <v>10.64</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>42.57</v>

</xml_diff>